<commit_message>
Finalize Q2389 StatefulSet rollout schedule
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R61ffa2d592c44d10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R2d11eee06c634c15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34,7 +34,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF2C5E86"/>
+        <x:fgColor rgb="FF315D72"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -42,14 +42,14 @@
     <x:border/>
     <x:border>
       <x:bottom style="thin">
-        <x:color rgb="FFD7E2EA"/>
+        <x:color rgb="FFD6E0E5"/>
       </x:bottom>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -70,9 +70,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -277,14 +274,14 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="132" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="142" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="9" t="str">
+      <x:c r="A1" s="8" t="str">
         <x:v>模块</x:v>
       </x:c>
-      <x:c r="B1" s="9" t="str">
+      <x:c r="B1" s="8" t="str">
         <x:v>规格内容</x:v>
       </x:c>
     </x:row>
@@ -293,7 +290,7 @@
         <x:v>任务ID</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
-        <x:v>statefulset_partition_rollout_review</x:v>
+        <x:v>statefulset_partition_rollout_schedule</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -309,7 +306,7 @@
         <x:v>辅助工具</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>kubectl1.32.6内置Kustomize、PowerShell7、Ruby3.3、UTF-8文本编辑器、CSV与JSON查看器</x:v>
+        <x:v>kubectl1.32.6内置Kustomize、PowerShell7、UTF-8文本编辑器、CSV与JSON查看器</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -317,7 +314,7 @@
         <x:v>输入来源</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>时序存储平台发布团队提供的合成阶段合同、探针样本和起始StatefulSet清单</x:v>
+        <x:v>时序存储平台发布值班提供的升级合同、现行StatefulSet清单和近期维护窗副本启动观测</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -333,7 +330,7 @@
         <x:v>原始输入文件</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>input_data/rollout_contract.json、input_data/ordinal_probes.csv、input_data/starter/statefulset.yaml和input_data/README.md</x:v>
+        <x:v>input_data/rollout_contract.json、input_data/ordinal_observations.csv、input_data/starter/statefulset.yaml和input_data/README.md</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -341,7 +338,7 @@
         <x:v>目标输出文件</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>output/kustomize、output/results、output/commands、output/run_release_review.rb、output/tools和output/README.md</x:v>
+        <x:v>output/kustomize、output/results、output/commands和output/README.md</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -349,7 +346,7 @@
         <x:v>核心操作链</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>核对阶段合同与样本→整理基础Service和StatefulSet→建立阶段覆盖层→构建四阶段清单→提取清单字段→归并探针样本→形成阶段结论→准备回退检查表</x:v>
+        <x:v>核对升级合同与历史观测→整理基础Service和StatefulSet→建立阶段覆盖层→构建四阶段候选清单→提取清单字段→整理历史观测→安排阶段→准备回退材料</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -370,58 +367,66 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="5" t="str">
-        <x:v>探针样本口径</x:v>
+        <x:v>清单台账</x:v>
       </x:c>
       <x:c r="B12" s="5" t="str">
-        <x:v>按phase与ordinal读取样本，startup_pass和ready均为true时记为SAMPLE_READY，其余记为SAMPLE_FAILED</x:v>
+        <x:v>manifest_ledger.csv记录四阶段镜像、partition、探针参数、卷保留字段和对象关系</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="5" t="str">
-        <x:v>阶段结论口径</x:v>
+        <x:v>历史观测</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>按合同列出的序号顺序收集样本，全部通过时为SAMPLE_CLEAR，出现失败样本时为SAMPLE_HOLD并记录首个失败序号</x:v>
+        <x:v>ordinal_observation_review.csv保留输入观测，startup_pass和ready均为true时记为READY，否则记为NOT_READY</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>回退清单口径</x:v>
+        <x:v>阶段排期</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>保留合同中的步骤、动作、前置条件和待收集材料，维护窗前execution_status统一为NOT_EXECUTED</x:v>
+        <x:v>按合同指定的序号整理观测，canary为PROCEED，promote为HOLD，rollback为READY_IF_APPROVED</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="5" t="str">
-        <x:v>结论范围</x:v>
+        <x:v>回退材料</x:v>
       </x:c>
       <x:c r="B15" s="5" t="str">
-        <x:v>本地清单与已有样本用于发布前判断，集群变更、控制器状态和PVC状态留待审批后的维护窗确认</x:v>
+        <x:v>rollback_checklist.csv保留合同中的步骤、动作、前提和待收集材料，维护窗前execution_status为PENDING</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>结论边界</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>四阶段清单均可由kubectl构建，清单字段与合同一致，8条样本完整归并，三阶段结论正确，5项回退检查连续且未执行</x:v>
+        <x:v>候选清单与历史观测用于维护窗排期，不代表本次集群变更、控制器动作或PVC状态已经发生</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="5" t="str">
+        <x:v>完成条件</x:v>
+      </x:c>
+      <x:c r="B17" s="5" t="str">
+        <x:v>四阶段清单可由kubectl构建，清单字段与合同一致，8条观测完整归并，三阶段排期正确，5项回退检查连续且状态为PENDING</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="5" t="str">
         <x:v>可验证点</x:v>
       </x:c>
-      <x:c r="B17" s="5" t="str">
-        <x:v>对象种类与名称、选择器闭合、镜像、partition、探针参数、卷保留字段、样本覆盖、阶段结论、回退步骤和复核摘要</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="6" t="str">
+      <x:c r="B18" s="5" t="str">
+        <x:v>对象种类与名称、选择器闭合、镜像、partition、探针参数、卷保留字段、观测覆盖、阶段排期、回退步骤和现场边界</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="6" t="str">
         <x:v>不适合作为评分点的内容</x:v>
       </x:c>
-      <x:c r="B18" s="6" t="str">
-        <x:v>YAML键序、文档顺序、注释、辅助标签、CSV行序、JSON缩进、临时目录和说明文字风格</x:v>
+      <x:c r="B19" s="6" t="str">
+        <x:v>YAML键序、文档顺序、注释、辅助标签、CSV行序、临时目录和说明文字风格</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>